<commit_message>
feat(payroll): mesai 1.5x ve eksik saat 1.0x formulu tum sisteme uygulandi
</commit_message>
<xml_diff>
--- a/pdks_eylul_gunluk_calisma_saatleri.xlsx
+++ b/pdks_eylul_gunluk_calisma_saatleri.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eylul_2026_Saatler" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_2026_Saatler" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -603,7 +603,7 @@
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>01.09
-Salı</t>
+Sal</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1869,44 +1869,44 @@
       </c>
       <c r="D17" s="6" t="n"/>
       <c r="E17" s="7" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="F17" s="8" t="n">
-        <v>7.5</v>
+        <v>10.5</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="G17" s="6" t="n"/>
       <c r="H17" s="6" t="n"/>
       <c r="I17" s="9" t="n"/>
-      <c r="J17" s="8" t="n">
-        <v>7.5</v>
+      <c r="J17" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="M17" s="8" t="n">
-        <v>7.5</v>
+        <v>10</v>
+      </c>
+      <c r="M17" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="N17" s="6" t="n"/>
       <c r="O17" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="P17" s="9" t="n"/>
       <c r="Q17" s="6" t="n"/>
       <c r="R17" s="6" t="n"/>
-      <c r="S17" s="8" t="n">
-        <v>7.5</v>
+      <c r="S17" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="T17" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="U17" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="V17" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="W17" s="9" t="n"/>
       <c r="X17" s="6" t="n"/>
@@ -1923,7 +1923,7 @@
         <v>11</v>
       </c>
       <c r="AI17" s="11" t="n">
-        <v>90</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1">
@@ -2722,57 +2722,57 @@
         </is>
       </c>
       <c r="D29" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="G29" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H29" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I29" s="9" t="n"/>
-      <c r="J29" s="8" t="n">
-        <v>6</v>
+      <c r="J29" s="7" t="n">
+        <v>8</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="L29" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M29" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="N29" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="O29" s="7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P29" s="9" t="n"/>
       <c r="Q29" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="S29" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="T29" s="8" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="U29" s="8" t="n">
-        <v>7.5</v>
+        <v>10</v>
+      </c>
+      <c r="S29" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="T29" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="U29" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="V29" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="W29" s="9" t="n"/>
       <c r="X29" s="6" t="n"/>
@@ -2789,7 +2789,7 @@
         <v>17</v>
       </c>
       <c r="AI29" s="11" t="n">
-        <v>138</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" ht="19" customHeight="1">
@@ -2983,50 +2983,50 @@
         </is>
       </c>
       <c r="D32" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F32" s="14" t="n"/>
       <c r="G32" s="14" t="n"/>
       <c r="H32" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I32" s="9" t="n"/>
-      <c r="J32" s="8" t="n">
-        <v>6.5</v>
+      <c r="J32" s="7" t="n">
+        <v>8.5</v>
       </c>
       <c r="K32" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="L32" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M32" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="N32" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="O32" s="8" t="n">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="O32" s="7" t="n">
+        <v>8</v>
       </c>
       <c r="P32" s="9" t="n"/>
       <c r="Q32" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R32" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="S32" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="T32" s="8" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="U32" s="8" t="n">
-        <v>7.5</v>
+        <v>10</v>
+      </c>
+      <c r="S32" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="T32" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="U32" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="V32" s="14" t="n"/>
       <c r="W32" s="9" t="n"/>
@@ -3044,7 +3044,7 @@
         <v>14</v>
       </c>
       <c r="AI32" s="11" t="n">
-        <v>108</v>
+        <v>136</v>
       </c>
     </row>
     <row r="33" ht="19" customHeight="1">
@@ -5379,42 +5379,42 @@
       <c r="G63" s="6" t="n"/>
       <c r="H63" s="6" t="n"/>
       <c r="I63" s="9" t="n"/>
-      <c r="J63" s="8" t="n">
-        <v>6.5</v>
+      <c r="J63" s="7" t="n">
+        <v>8.5</v>
       </c>
       <c r="K63" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="L63" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M63" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="N63" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="O63" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="P63" s="9" t="n"/>
       <c r="Q63" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="R63" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="S63" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="T63" s="8" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="U63" s="8" t="n">
-        <v>7.5</v>
+        <v>10</v>
+      </c>
+      <c r="S63" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="T63" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="U63" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="V63" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="W63" s="9" t="n"/>
       <c r="X63" s="6" t="n"/>
@@ -5431,7 +5431,7 @@
         <v>12</v>
       </c>
       <c r="AI63" s="11" t="n">
-        <v>95</v>
+        <v>119</v>
       </c>
     </row>
     <row r="64" ht="19" customHeight="1">
@@ -7254,57 +7254,57 @@
         </is>
       </c>
       <c r="D87" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="E87" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F87" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="G87" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H87" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I87" s="9" t="n"/>
-      <c r="J87" s="8" t="n">
-        <v>6</v>
+      <c r="J87" s="7" t="n">
+        <v>8</v>
       </c>
       <c r="K87" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="L87" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M87" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="N87" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="O87" s="7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P87" s="9" t="n"/>
       <c r="Q87" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="R87" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="S87" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="T87" s="8" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="U87" s="8" t="n">
-        <v>7.5</v>
+        <v>10</v>
+      </c>
+      <c r="S87" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="T87" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="U87" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="V87" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="W87" s="9" t="n"/>
       <c r="X87" s="6" t="n"/>
@@ -7321,7 +7321,7 @@
         <v>17</v>
       </c>
       <c r="AI87" s="11" t="n">
-        <v>138</v>
+        <v>172</v>
       </c>
     </row>
     <row r="88" ht="19" customHeight="1">
@@ -8380,57 +8380,57 @@
         </is>
       </c>
       <c r="D101" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="E101" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F101" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="G101" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H101" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I101" s="9" t="n"/>
-      <c r="J101" s="8" t="n">
-        <v>6.5</v>
+      <c r="J101" s="7" t="n">
+        <v>8.5</v>
       </c>
       <c r="K101" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="L101" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M101" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="N101" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="O101" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="P101" s="9" t="n"/>
       <c r="Q101" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="R101" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="S101" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="T101" s="8" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="U101" s="8" t="n">
-        <v>7.5</v>
+        <v>10</v>
+      </c>
+      <c r="S101" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="T101" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="U101" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="V101" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="W101" s="9" t="n"/>
       <c r="X101" s="6" t="n"/>
@@ -8447,7 +8447,7 @@
         <v>17</v>
       </c>
       <c r="AI101" s="11" t="n">
-        <v>138</v>
+        <v>172</v>
       </c>
     </row>
     <row r="102" ht="19" customHeight="1">
@@ -8626,25 +8626,25 @@
           <t>BALIK KESİM</t>
         </is>
       </c>
-      <c r="D104" s="8" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="E104" s="8" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="F104" s="8" t="n">
-        <v>7.5</v>
+      <c r="D104" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E104" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="F104" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="G104" s="14" t="n"/>
       <c r="H104" s="14" t="n"/>
       <c r="I104" s="7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J104" s="7" t="n">
         <v>13.5</v>
       </c>
-      <c r="K104" s="8" t="n">
-        <v>7.5</v>
+      <c r="K104" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="L104" s="7" t="n">
         <v>14</v>
@@ -8665,14 +8665,14 @@
       <c r="R104" s="7" t="n">
         <v>17.5</v>
       </c>
-      <c r="S104" s="8" t="n">
-        <v>7.5</v>
+      <c r="S104" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="T104" s="14" t="n"/>
       <c r="U104" s="14" t="n"/>
       <c r="V104" s="14" t="n"/>
-      <c r="W104" s="8" t="n">
-        <v>7</v>
+      <c r="W104" s="7" t="n">
+        <v>9</v>
       </c>
       <c r="X104" s="14" t="n"/>
       <c r="Y104" s="14" t="n"/>
@@ -8688,7 +8688,7 @@
         <v>14</v>
       </c>
       <c r="AI104" s="11" t="n">
-        <v>151.5</v>
+        <v>165.5</v>
       </c>
     </row>
     <row r="105" ht="19" customHeight="1">
@@ -9133,7 +9133,7 @@
         <v>14.5</v>
       </c>
       <c r="E111" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="F111" s="7" t="n">
         <v>13.5</v>
@@ -9142,14 +9142,14 @@
         <v>13</v>
       </c>
       <c r="H111" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="I111" s="9" t="n"/>
-      <c r="J111" s="8" t="n">
-        <v>7</v>
+      <c r="J111" s="7" t="n">
+        <v>9</v>
       </c>
       <c r="K111" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="L111" s="7" t="n">
         <v>12.5</v>
@@ -9162,26 +9162,26 @@
         <v>14.5</v>
       </c>
       <c r="P111" s="9" t="n"/>
-      <c r="Q111" s="8" t="n">
-        <v>7.5</v>
+      <c r="Q111" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="R111" s="7" t="n">
         <v>12.5</v>
       </c>
       <c r="S111" s="7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="T111" s="7" t="n">
         <v>12</v>
       </c>
       <c r="U111" s="7" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="V111" s="8" t="n">
-        <v>7.5</v>
+        <v>10.5</v>
+      </c>
+      <c r="V111" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="W111" s="8" t="n">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="X111" s="6" t="n"/>
       <c r="Y111" s="6" t="n"/>
@@ -9197,7 +9197,7 @@
         <v>17</v>
       </c>
       <c r="AI111" s="11" t="n">
-        <v>172</v>
+        <v>190</v>
       </c>
     </row>
     <row r="112" ht="19" customHeight="1">
@@ -9604,57 +9604,57 @@
         </is>
       </c>
       <c r="D117" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="E117" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F117" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="G117" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H117" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I117" s="9" t="n"/>
-      <c r="J117" s="8" t="n">
-        <v>6</v>
+      <c r="J117" s="7" t="n">
+        <v>8</v>
       </c>
       <c r="K117" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="L117" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M117" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="N117" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="O117" s="7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P117" s="9" t="n"/>
       <c r="Q117" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="R117" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="S117" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="T117" s="8" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="U117" s="8" t="n">
-        <v>7.5</v>
+        <v>10</v>
+      </c>
+      <c r="S117" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="T117" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="U117" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="V117" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="W117" s="9" t="n"/>
       <c r="X117" s="6" t="n"/>
@@ -9671,7 +9671,7 @@
         <v>17</v>
       </c>
       <c r="AI117" s="11" t="n">
-        <v>138</v>
+        <v>172</v>
       </c>
     </row>
     <row r="118" ht="19" customHeight="1">
@@ -10241,37 +10241,37 @@
           <t>BALIK KESİM</t>
         </is>
       </c>
-      <c r="D125" s="8" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="E125" s="8" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="F125" s="8" t="n">
-        <v>7.5</v>
+      <c r="D125" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E125" s="7" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="F125" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="G125" s="7" t="n">
         <v>12.5</v>
       </c>
       <c r="H125" s="6" t="n"/>
       <c r="I125" s="7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="J125" s="6" t="n"/>
-      <c r="K125" s="8" t="n">
-        <v>7.5</v>
+      <c r="K125" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="L125" s="6" t="n"/>
       <c r="M125" s="7" t="n">
         <v>13.5</v>
       </c>
-      <c r="N125" s="8" t="n">
-        <v>7.5</v>
+      <c r="N125" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="O125" s="6" t="n"/>
       <c r="P125" s="9" t="n"/>
-      <c r="Q125" s="8" t="n">
-        <v>7.5</v>
+      <c r="Q125" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="R125" s="6" t="n"/>
       <c r="S125" s="6" t="n"/>
@@ -10293,7 +10293,7 @@
         <v>9</v>
       </c>
       <c r="AI125" s="11" t="n">
-        <v>80</v>
+        <v>94</v>
       </c>
     </row>
     <row r="126" ht="19" customHeight="1">
@@ -19952,51 +19952,51 @@
         </is>
       </c>
       <c r="D251" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="E251" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F251" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="G251" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H251" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I251" s="9" t="n"/>
-      <c r="J251" s="8" t="n">
-        <v>6</v>
+      <c r="J251" s="7" t="n">
+        <v>8</v>
       </c>
       <c r="K251" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="L251" s="6" t="n"/>
       <c r="M251" s="6" t="n"/>
       <c r="N251" s="6" t="n"/>
       <c r="O251" s="7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="P251" s="9" t="n"/>
       <c r="Q251" s="7" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="R251" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="S251" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="T251" s="8" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="U251" s="8" t="n">
-        <v>7.5</v>
+        <v>10</v>
+      </c>
+      <c r="S251" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="T251" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="U251" s="7" t="n">
+        <v>9.5</v>
       </c>
       <c r="V251" s="7" t="n">
-        <v>9.5</v>
+        <v>11.5</v>
       </c>
       <c r="W251" s="9" t="n"/>
       <c r="X251" s="6" t="n"/>
@@ -20013,7 +20013,7 @@
         <v>14</v>
       </c>
       <c r="AI251" s="11" t="n">
-        <v>112.5</v>
+        <v>140.5</v>
       </c>
     </row>
     <row r="252" ht="19" customHeight="1">

</xml_diff>